<commit_message>
actualización links e imagen de muestra bd
</commit_message>
<xml_diff>
--- a/links de interes.xlsx
+++ b/links de interes.xlsx
@@ -9,7 +9,7 @@
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913" iterateDelta="1E-4"/>
+  <calcPr calcId="162913"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="84">
   <si>
     <t>Enlace</t>
   </si>
@@ -259,6 +259,18 @@
   </si>
   <si>
     <t>Aprender git jugado</t>
+  </si>
+  <si>
+    <t>https://www.bcn.cl/leychile/navegar?idNorma=1209272</t>
+  </si>
+  <si>
+    <t>La Ley 21.719 es la nueva normativa chilena de Protección de Datos Personales.</t>
+  </si>
+  <si>
+    <t>https://dbdiagram.io/home</t>
+  </si>
+  <si>
+    <t>para la creación de diagramas</t>
   </si>
 </sst>
 </file>
@@ -282,12 +294,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF92D050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -303,13 +321,15 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
@@ -591,7 +611,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="B2:C43"/>
+  <dimension ref="B2:C45"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="64.28515625" bestFit="1" customWidth="1"/>
@@ -932,6 +952,22 @@
       </c>
       <c r="C43" t="s">
         <v>60</v>
+      </c>
+    </row>
+    <row r="44" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B44" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="C44" s="5" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="45" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B45" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="C45" t="s">
+        <v>83</v>
       </c>
     </row>
   </sheetData>
@@ -977,8 +1013,10 @@
     <hyperlink ref="B36" r:id="rId39"/>
     <hyperlink ref="B13" r:id="rId40"/>
     <hyperlink ref="B14" r:id="rId41"/>
+    <hyperlink ref="B44" r:id="rId42"/>
+    <hyperlink ref="B45" r:id="rId43"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId42"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId44"/>
 </worksheet>
 </file>
</xml_diff>